<commit_message>
save 02 07 2026
</commit_message>
<xml_diff>
--- a/# четверть_#_полезные ссылки для тестирования сайтов рассылок.xlsx
+++ b/# четверть_#_полезные ссылки для тестирования сайтов рассылок.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexServHW\Desktop\GB_Developer_Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F135F3B-8B13-4103-B34F-B7299D006946}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC4FC914-BC1F-41CF-B2C0-C4DEA99E5926}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10770" yWindow="-15420" windowWidth="23250" windowHeight="12450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-8820" yWindow="-16920" windowWidth="23250" windowHeight="12450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="12" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Урок 1 часть 1</t>
   </si>
@@ -42,6 +42,12 @@
     <t>Вот одна галочка не зелененькая, а желтенькая именно потому что нет ссылки на отписку.
 По этому критерию ранжируются рассылки и им выставляется соответствующий рейтинг.
 Без ссылки на отписку рейтинг понижается с каждым письмом.</t>
+  </si>
+  <si>
+    <t>CrowdSec Web UI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/TheDuffman85/crowdsec-web-ui </t>
   </si>
 </sst>
 </file>
@@ -434,7 +440,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:V4"/>
+  <dimension ref="A2:V5"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36" style="1" customWidth="1"/>
@@ -505,12 +511,21 @@
         <v>1</v>
       </c>
     </row>
+    <row r="5" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="C4" r:id="rId1" xr:uid="{E8D62272-8175-47AE-9712-C94739EB9ACC}"/>
+    <hyperlink ref="C5" r:id="rId2" xr:uid="{14C24C52-D807-4F34-9DBD-8A3F76FDA123}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId2"/>
+  <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
save 16 07 2025
</commit_message>
<xml_diff>
--- a/# четверть_#_полезные ссылки для тестирования сайтов рассылок.xlsx
+++ b/# четверть_#_полезные ссылки для тестирования сайтов рассылок.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexServHW\Desktop\GB_Developer_Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC4FC914-BC1F-41CF-B2C0-C4DEA99E5926}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4658BA1-53CC-4E96-8A2A-AA82C82178B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-8820" yWindow="-16920" windowWidth="23250" windowHeight="12450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12015" yWindow="-17835" windowWidth="23010" windowHeight="12210" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="12" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Урок 1 часть 1</t>
   </si>
@@ -48,18 +48,32 @@
   </si>
   <si>
     <t xml:space="preserve">https://github.com/TheDuffman85/crowdsec-web-ui </t>
+  </si>
+  <si>
+    <t>reg.ru</t>
+  </si>
+  <si>
+    <t>cert</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -124,9 +138,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -137,23 +151,26 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -440,7 +457,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:V5"/>
+  <dimension ref="A2:V7"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36" style="1" customWidth="1"/>
@@ -519,8 +536,18 @@
         <v>5</v>
       </c>
     </row>
+    <row r="6" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="C6" s="11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="C7" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
-  <phoneticPr fontId="3" type="noConversion"/>
+  <phoneticPr fontId="4" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="C4" r:id="rId1" xr:uid="{E8D62272-8175-47AE-9712-C94739EB9ACC}"/>
     <hyperlink ref="C5" r:id="rId2" xr:uid="{14C24C52-D807-4F34-9DBD-8A3F76FDA123}"/>

</xml_diff>

<commit_message>
save 31 07 2026
</commit_message>
<xml_diff>
--- a/# четверть_#_полезные ссылки для тестирования сайтов рассылок.xlsx
+++ b/# четверть_#_полезные ссылки для тестирования сайтов рассылок.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexServHW\Desktop\GB_Developer_Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4658BA1-53CC-4E96-8A2A-AA82C82178B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ABD9C81-0398-4BC2-AF3C-CCB218B09A82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12015" yWindow="-17835" windowWidth="23010" windowHeight="12210" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5985" yWindow="-14175" windowWidth="23010" windowHeight="11130" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="12" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Урок 1 часть 1</t>
   </si>
@@ -53,7 +53,22 @@
     <t>reg.ru</t>
   </si>
   <si>
-    <t>cert</t>
+    <t>sqlguardjs</t>
+  </si>
+  <si>
+    <t>let's encrypt</t>
+  </si>
+  <si>
+    <t>Регистрация доменов</t>
+  </si>
+  <si>
+    <t>Получение SSL сертификата</t>
+  </si>
+  <si>
+    <t>SQL инъекции</t>
+  </si>
+  <si>
+    <t>Наблюдение за сервисами (над kuberneties)</t>
   </si>
 </sst>
 </file>
@@ -457,7 +472,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:V7"/>
+  <dimension ref="A2:V8"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36" style="1" customWidth="1"/>
@@ -532,25 +547,42 @@
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="10" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A6" s="11" t="s">
+        <v>6</v>
+      </c>
       <c r="C6" s="11" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A7" s="11" t="s">
+        <v>8</v>
+      </c>
       <c r="C7" s="11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A8" s="11" t="s">
         <v>7</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="C4" r:id="rId1" xr:uid="{E8D62272-8175-47AE-9712-C94739EB9ACC}"/>
-    <hyperlink ref="C5" r:id="rId2" xr:uid="{14C24C52-D807-4F34-9DBD-8A3F76FDA123}"/>
+    <hyperlink ref="D5" r:id="rId2" xr:uid="{14C24C52-D807-4F34-9DBD-8A3F76FDA123}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId3"/>

</xml_diff>

<commit_message>
save 13 08 2026
</commit_message>
<xml_diff>
--- a/# четверть_#_полезные ссылки для тестирования сайтов рассылок.xlsx
+++ b/# четверть_#_полезные ссылки для тестирования сайтов рассылок.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexServHW\Desktop\GB_Developer_Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ABD9C81-0398-4BC2-AF3C-CCB218B09A82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAAA8F15-2818-4294-8D34-218367D79251}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5985" yWindow="-14175" windowWidth="23010" windowHeight="11130" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="24" yWindow="1104" windowWidth="23016" windowHeight="11136" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="12" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>Урок 1 часть 1</t>
   </si>
@@ -69,18 +69,83 @@
   </si>
   <si>
     <t>Наблюдение за сервисами (над kuberneties)</t>
+  </si>
+  <si>
+    <t>infisical</t>
+  </si>
+  <si>
+    <t>Хранение секретов</t>
+  </si>
+  <si>
+    <t>`https://yandex.ru/safety/</t>
+  </si>
+  <si>
+    <t>проверка безопасности сайта</t>
+  </si>
+  <si>
+    <t>quasar</t>
+  </si>
+  <si>
+    <t>`https://www.syncfusion.com/javascript-ui-controls/js-data-grid</t>
+  </si>
+  <si>
+    <t>красивые вебтаблицы</t>
+  </si>
+  <si>
+    <t>`https://handsontable.com/</t>
+  </si>
+  <si>
+    <t>красивые вебтаблицы в виде xls</t>
+  </si>
+  <si>
+    <t>`https://echarts.apache.org/en/index.html</t>
+  </si>
+  <si>
+    <t>Apache echarts</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -153,9 +218,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -166,23 +231,35 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -472,7 +549,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:V8"/>
+  <dimension ref="A2:V14"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36" style="1" customWidth="1"/>
@@ -578,8 +655,53 @@
         <v>11</v>
       </c>
     </row>
+    <row r="9" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="13" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13" s="14" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C14" s="15" t="s">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
-  <phoneticPr fontId="4" type="noConversion"/>
+  <phoneticPr fontId="8" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="C4" r:id="rId1" xr:uid="{E8D62272-8175-47AE-9712-C94739EB9ACC}"/>
     <hyperlink ref="D5" r:id="rId2" xr:uid="{14C24C52-D807-4F34-9DBD-8A3F76FDA123}"/>

</xml_diff>

<commit_message>
save 24 08 2026
</commit_message>
<xml_diff>
--- a/# четверть_#_полезные ссылки для тестирования сайтов рассылок.xlsx
+++ b/# четверть_#_полезные ссылки для тестирования сайтов рассылок.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexServHW\Desktop\GB_Developer_Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAAA8F15-2818-4294-8D34-218367D79251}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{656028D9-5355-4705-B3B2-DFF626526C56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="24" yWindow="1104" windowWidth="23016" windowHeight="11136" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="12" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>Урок 1 часть 1</t>
   </si>
@@ -102,18 +102,32 @@
   </si>
   <si>
     <t>Apache echarts</t>
+  </si>
+  <si>
+    <t>`https://github.com/exceljs/exceljs</t>
+  </si>
+  <si>
+    <t>Exceljs</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+  <fonts count="11" x14ac:knownFonts="1">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -218,9 +232,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -231,23 +245,26 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -549,7 +566,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:V14"/>
+  <dimension ref="A2:V15"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36" style="1" customWidth="1"/>
@@ -700,8 +717,16 @@
         <v>23</v>
       </c>
     </row>
+    <row r="15" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C15" s="16" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
-  <phoneticPr fontId="8" type="noConversion"/>
+  <phoneticPr fontId="9" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="C4" r:id="rId1" xr:uid="{E8D62272-8175-47AE-9712-C94739EB9ACC}"/>
     <hyperlink ref="D5" r:id="rId2" xr:uid="{14C24C52-D807-4F34-9DBD-8A3F76FDA123}"/>

</xml_diff>

<commit_message>
save 01 09 2026
</commit_message>
<xml_diff>
--- a/# четверть_#_полезные ссылки для тестирования сайтов рассылок.xlsx
+++ b/# четверть_#_полезные ссылки для тестирования сайтов рассылок.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexServHW\Desktop\GB_Developer_Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{656028D9-5355-4705-B3B2-DFF626526C56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4A0E599-0E88-4963-81A2-C01ED23447DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3480" yWindow="-16140" windowWidth="26445" windowHeight="13470" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="12" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
   <si>
     <t>Урок 1 часть 1</t>
   </si>
@@ -108,18 +108,102 @@
   </si>
   <si>
     <t>Exceljs</t>
+  </si>
+  <si>
+    <t>`https://habr.com/ru/companies/ru_mts/articles/967598/</t>
+  </si>
+  <si>
+    <t>приблуда для удаленного подключения к пк</t>
+  </si>
+  <si>
+    <t>`https://technitium.com/dns/</t>
+  </si>
+  <si>
+    <t>DNS server opensource</t>
+  </si>
+  <si>
+    <t>Onlyoffice</t>
+  </si>
+  <si>
+    <t>MS Office для Linux</t>
+  </si>
+  <si>
+    <t>`https://amplicode.ru/?utm_source=habr&amp;utm_medium=referral&amp;utm_campaign=haulmont-blog</t>
+  </si>
+  <si>
+    <t>Java Spring AI helper</t>
+  </si>
+  <si>
+    <t>Talos (над kuberneties)</t>
+  </si>
+  <si>
+    <t>`https://www.siderolabs.com/talos-linux</t>
+  </si>
+  <si>
+    <t>`https://n8n.io/case-studies/huel/</t>
+  </si>
+  <si>
+    <t>n8n (автоматизация процессов)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+  <fonts count="17" x14ac:knownFonts="1">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -232,9 +316,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -245,23 +329,41 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="14" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -566,7 +668,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:V15"/>
+  <dimension ref="A2:V21"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36" style="1" customWidth="1"/>
@@ -725,8 +827,56 @@
         <v>25</v>
       </c>
     </row>
+    <row r="16" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C16" s="17" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17" s="18" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" s="19" t="s">
+        <v>30</v>
+      </c>
+      <c r="C18" s="19" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C19" s="20" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C20" s="21" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C21" s="22" t="s">
+        <v>37</v>
+      </c>
+    </row>
   </sheetData>
-  <phoneticPr fontId="9" type="noConversion"/>
+  <phoneticPr fontId="15" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="C4" r:id="rId1" xr:uid="{E8D62272-8175-47AE-9712-C94739EB9ACC}"/>
     <hyperlink ref="D5" r:id="rId2" xr:uid="{14C24C52-D807-4F34-9DBD-8A3F76FDA123}"/>

</xml_diff>

<commit_message>
save 04 09 2026
</commit_message>
<xml_diff>
--- a/# четверть_#_полезные ссылки для тестирования сайтов рассылок.xlsx
+++ b/# четверть_#_полезные ссылки для тестирования сайтов рассылок.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexServHW\Desktop\GB_Developer_Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4A0E599-0E88-4963-81A2-C01ED23447DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{870A7E86-91FB-4CCE-A221-8210C58E4391}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3480" yWindow="-16140" windowWidth="26445" windowHeight="13470" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8940" yWindow="-17025" windowWidth="23250" windowHeight="12450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="12" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
   <si>
     <t>Урок 1 часть 1</t>
   </si>
@@ -144,18 +144,34 @@
   </si>
   <si>
     <t>n8n (автоматизация процессов)</t>
+  </si>
+  <si>
+    <t>https://vast.ai/pricing#gpu-grid - аренда серверов с видео-картами
+https://unsloth.ai/ - загрузка и run нейронок локально (устанавливаем на арендованном сервере)
+Kilo Code для vscode - прописывам ssh для доступа к запущенной нейронке на рендованном сервере</t>
+  </si>
+  <si>
+    <t>Запуск нейронок на локально арендованном сервере</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="17" x14ac:knownFonts="1">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+  <fonts count="18" x14ac:knownFonts="1">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -316,9 +332,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -329,23 +345,26 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="14" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="15" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -668,7 +687,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:V21"/>
+  <dimension ref="A2:V22"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36" style="1" customWidth="1"/>
@@ -875,8 +894,16 @@
         <v>37</v>
       </c>
     </row>
+    <row r="22" spans="1:3" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A22" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="C22" s="23" t="s">
+        <v>39</v>
+      </c>
+    </row>
   </sheetData>
-  <phoneticPr fontId="15" type="noConversion"/>
+  <phoneticPr fontId="16" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="C4" r:id="rId1" xr:uid="{E8D62272-8175-47AE-9712-C94739EB9ACC}"/>
     <hyperlink ref="D5" r:id="rId2" xr:uid="{14C24C52-D807-4F34-9DBD-8A3F76FDA123}"/>

</xml_diff>